<commit_message>
Blueprint passes round 3; Phase 1 complete
</commit_message>
<xml_diff>
--- a/book/model/build/Ch40_funding.xlsx
+++ b/book/model/build/Ch40_funding.xlsx
@@ -723,7 +723,7 @@
     <row r="31">
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Build-along file Ch40_funding.xlsx: the companion model at the end of Chapter 40 (u09 Section 0.4 rows of Chapters 39 to 40; model version 1.4).</t>
+          <t>Build-along file Ch40_funding.xlsx: the companion model at the end of Chapter 40 (u09 Section 0.4 rows of Chapters 39 to 40; model version 1.5).</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
         </is>
       </c>
       <c r="F113" s="7" t="n">
-        <v>633.2559755427742</v>
+        <v>629.9496747784333</v>
       </c>
     </row>
     <row r="114">
@@ -3623,7 +3623,7 @@
         </is>
       </c>
       <c r="F114" s="7" t="n">
-        <v>221.8337675840513</v>
+        <v>224.6022195891398</v>
       </c>
     </row>
     <row r="185">
@@ -6172,7 +6172,7 @@
     <row r="298">
       <c r="D298" t="inlineStr">
         <is>
-          <t>Contract repayment profile at FC (share of debt)</t>
+          <t>Contract repayment profile at FC, A-loan, B-loan, commercial and standby (share of their amount; ECA in equal installments)</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -6199,82 +6199,82 @@
         <v>0</v>
       </c>
       <c r="P298" s="6" t="n">
-        <v>0.02446043211430804</v>
+        <v>0.01890095694428932</v>
       </c>
       <c r="Q298" s="6" t="n">
-        <v>0.02549563991993633</v>
+        <v>0.0202905789790784</v>
       </c>
       <c r="R298" s="6" t="n">
-        <v>0.02675152229066621</v>
+        <v>0.02200332954137934</v>
       </c>
       <c r="S298" s="6" t="n">
-        <v>0.02753984637468513</v>
+        <v>0.0230513965167324</v>
       </c>
       <c r="T298" s="6" t="n">
-        <v>0.0288066694390464</v>
+        <v>0.02478569830568763</v>
       </c>
       <c r="U298" s="6" t="n">
-        <v>0.02972536483920772</v>
+        <v>0.026031162687892</v>
       </c>
       <c r="V298" s="6" t="n">
-        <v>0.03166730192250924</v>
+        <v>0.02874437196072473</v>
       </c>
       <c r="W298" s="6" t="n">
-        <v>0.03263535190708168</v>
+        <v>0.03008036171890596</v>
       </c>
       <c r="X298" s="6" t="n">
-        <v>0.0317294685115491</v>
+        <v>0.0287176079977811</v>
       </c>
       <c r="Y298" s="6" t="n">
-        <v>0.03174439879630291</v>
+        <v>0.02863354718565791</v>
       </c>
       <c r="Z298" s="6" t="n">
-        <v>0.03305950431870376</v>
+        <v>0.03043907604633617</v>
       </c>
       <c r="AA298" s="6" t="n">
-        <v>0.03402426353926975</v>
+        <v>0.03176938173911321</v>
       </c>
       <c r="AB298" s="6" t="n">
-        <v>0.03564974851234601</v>
+        <v>0.03403191413177876</v>
       </c>
       <c r="AC298" s="6" t="n">
-        <v>0.03683076964636899</v>
+        <v>0.03568651766808281</v>
       </c>
       <c r="AD298" s="6" t="n">
-        <v>0.0402165127561107</v>
+        <v>0.0404984098748</v>
       </c>
       <c r="AE298" s="6" t="n">
-        <v>0.04194504016536777</v>
+        <v>0.04297859472667483</v>
       </c>
       <c r="AF298" s="6" t="n">
-        <v>0.04341654712966558</v>
+        <v>0.0450772391622633</v>
       </c>
       <c r="AG298" s="6" t="n">
-        <v>0.04422683953596448</v>
+        <v>0.04620125941456013</v>
       </c>
       <c r="AH298" s="6" t="n">
-        <v>0.0464470950071792</v>
+        <v>0.04939410723905355</v>
       </c>
       <c r="AI298" s="6" t="n">
-        <v>0.04781089882837024</v>
+        <v>0.05140402574797549</v>
       </c>
       <c r="AJ298" s="6" t="n">
-        <v>0.05011909730654722</v>
+        <v>0.05475917262981699</v>
       </c>
       <c r="AK298" s="6" t="n">
-        <v>0.05174136373715012</v>
+        <v>0.05717151219099544</v>
       </c>
       <c r="AL298" s="6" t="n">
-        <v>0.05486337334066368</v>
+        <v>0.06174196213781533</v>
       </c>
       <c r="AM298" s="6" t="n">
-        <v>0.05600370673381757</v>
+        <v>0.06420920211471677</v>
       </c>
       <c r="AN298" s="6" t="n">
-        <v>0.04620239321839347</v>
+        <v>0.05246029368361199</v>
       </c>
       <c r="AO298" s="6" t="n">
-        <v>0.04688685010878882</v>
+        <v>0.05093831965427672</v>
       </c>
       <c r="AP298" s="6" t="n">
         <v>0</v>
@@ -6355,7 +6355,7 @@
     <row r="299">
       <c r="D299" t="inlineStr">
         <is>
-          <t>COD re-sculpted repayment profile (share of debt at COD)</t>
+          <t>COD re-sculpted repayment profile, tranches other than ECA (share of their amount at COD)</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -6385,79 +6385,79 @@
         <v>0</v>
       </c>
       <c r="Q299" s="6" t="n">
-        <v>0.02492121667112088</v>
+        <v>0.01916933528318169</v>
       </c>
       <c r="R299" s="6" t="n">
-        <v>0.02664660047040042</v>
+        <v>0.02153568717143909</v>
       </c>
       <c r="S299" s="6" t="n">
-        <v>0.02759604458467765</v>
+        <v>0.02280073147930074</v>
       </c>
       <c r="T299" s="6" t="n">
-        <v>0.02888825064959648</v>
+        <v>0.02455871493656759</v>
       </c>
       <c r="U299" s="6" t="n">
-        <v>0.0296987112931962</v>
+        <v>0.02563708632237413</v>
       </c>
       <c r="V299" s="6" t="n">
-        <v>0.03105885768561841</v>
+        <v>0.02749943258581268</v>
       </c>
       <c r="W299" s="6" t="n">
-        <v>0.03277706730010246</v>
+        <v>0.02988602713814689</v>
       </c>
       <c r="X299" s="6" t="n">
-        <v>0.03427956112200796</v>
+        <v>0.03196578624060889</v>
       </c>
       <c r="Y299" s="6" t="n">
-        <v>0.03185352351247105</v>
+        <v>0.02841811790586881</v>
       </c>
       <c r="Z299" s="6" t="n">
-        <v>0.03335144112570533</v>
+        <v>0.0304704935092369</v>
       </c>
       <c r="AA299" s="6" t="n">
-        <v>0.03404882778677493</v>
+        <v>0.0314057361909549</v>
       </c>
       <c r="AB299" s="6" t="n">
-        <v>0.03570569600105964</v>
+        <v>0.0336946453904792</v>
       </c>
       <c r="AC299" s="6" t="n">
-        <v>0.03672091019892312</v>
+        <v>0.035095023088361</v>
       </c>
       <c r="AD299" s="6" t="n">
-        <v>0.0384689461355592</v>
+        <v>0.037532638887578</v>
       </c>
       <c r="AE299" s="6" t="n">
-        <v>0.04158438492613827</v>
+        <v>0.04195228966521355</v>
       </c>
       <c r="AF299" s="6" t="n">
-        <v>0.04382240991310483</v>
+        <v>0.04512050681432067</v>
       </c>
       <c r="AG299" s="6" t="n">
-        <v>0.04413949061350413</v>
+        <v>0.0455258173841402</v>
       </c>
       <c r="AH299" s="6" t="n">
-        <v>0.04642087223316833</v>
+        <v>0.04877459666480332</v>
       </c>
       <c r="AI299" s="6" t="n">
-        <v>0.04787232137396746</v>
+        <v>0.05088398599671974</v>
       </c>
       <c r="AJ299" s="6" t="n">
-        <v>0.0502195640539474</v>
+        <v>0.05426186417991957</v>
       </c>
       <c r="AK299" s="6" t="n">
-        <v>0.05170891802557741</v>
+        <v>0.05645632607798638</v>
       </c>
       <c r="AL299" s="6" t="n">
-        <v>0.0541382044749565</v>
+        <v>0.05999457970251743</v>
       </c>
       <c r="AM299" s="6" t="n">
-        <v>0.05666149382313952</v>
+        <v>0.06370476161482863</v>
       </c>
       <c r="AN299" s="6" t="n">
-        <v>0.05940104456083106</v>
+        <v>0.06773633457954874</v>
       </c>
       <c r="AO299" s="6" t="n">
-        <v>0.05801564146445255</v>
+        <v>0.06591948119009279</v>
       </c>
       <c r="AP299" s="6" t="n">
         <v>0</v>
@@ -6589,76 +6589,76 @@
         <v>0</v>
       </c>
       <c r="X300" s="6" t="n">
-        <v>0.01109281170584355</v>
+        <v>0.006829353124439196</v>
       </c>
       <c r="Y300" s="6" t="n">
-        <v>0.01611192821167361</v>
+        <v>0.01114889840603912</v>
       </c>
       <c r="Z300" s="6" t="n">
-        <v>0.01761625979950614</v>
+        <v>0.01330764450807491</v>
       </c>
       <c r="AA300" s="6" t="n">
-        <v>0.01756090365083943</v>
+        <v>0.01349709315044692</v>
       </c>
       <c r="AB300" s="6" t="n">
-        <v>0.01888075218483377</v>
+        <v>0.01557318313269935</v>
       </c>
       <c r="AC300" s="6" t="n">
-        <v>0.01890834059725892</v>
+        <v>0.01606185219857658</v>
       </c>
       <c r="AD300" s="6" t="n">
-        <v>0.02002427691925613</v>
+        <v>0.01799374116666692</v>
       </c>
       <c r="AE300" s="6" t="n">
-        <v>0.0220425537786885</v>
+        <v>0.02144458336133691</v>
       </c>
       <c r="AF300" s="6" t="n">
-        <v>0.02353641033974216</v>
+        <v>0.02402062562945583</v>
       </c>
       <c r="AG300" s="6" t="n">
-        <v>0.02376200405504096</v>
+        <v>0.02440292916342236</v>
       </c>
       <c r="AH300" s="6" t="n">
-        <v>0.02514405847890659</v>
+        <v>0.02690633991137525</v>
       </c>
       <c r="AI300" s="6" t="n">
-        <v>0.02522742917041925</v>
+        <v>0.02770096226699488</v>
       </c>
       <c r="AJ300" s="6" t="n">
-        <v>0.02649633835540665</v>
+        <v>0.03014523344881054</v>
       </c>
       <c r="AK300" s="6" t="n">
-        <v>0.02661192441658703</v>
+        <v>0.03102163191978114</v>
       </c>
       <c r="AL300" s="6" t="n">
-        <v>0.02773427333606693</v>
+        <v>0.03337597519823951</v>
       </c>
       <c r="AM300" s="6" t="n">
-        <v>0.02874043283146949</v>
+        <v>0.03565166194055328</v>
       </c>
       <c r="AN300" s="6" t="n">
-        <v>0.0299976714643956</v>
+        <v>0.03831792958389687</v>
       </c>
       <c r="AO300" s="6" t="n">
-        <v>0.02696870435180381</v>
+        <v>0.03477191605870274</v>
       </c>
       <c r="AP300" s="6" t="n">
-        <v>0.09367671694203662</v>
+        <v>0.09492419694885829</v>
       </c>
       <c r="AQ300" s="6" t="n">
-        <v>0.08896197241765595</v>
+        <v>0.08594938105303467</v>
       </c>
       <c r="AR300" s="6" t="n">
-        <v>0.09361458458293083</v>
+        <v>0.0904413102207277</v>
       </c>
       <c r="AS300" s="6" t="n">
-        <v>0.09576367135514924</v>
+        <v>0.09251459827539707</v>
       </c>
       <c r="AT300" s="6" t="n">
-        <v>0.1003452008485892</v>
+        <v>0.0969374640921163</v>
       </c>
       <c r="AU300" s="6" t="n">
-        <v>0.1211807802058968</v>
+        <v>0.1170614952403567</v>
       </c>
       <c r="AV300" s="6" t="n">
         <v>0</v>
@@ -6748,82 +6748,82 @@
         <v>0</v>
       </c>
       <c r="P301" s="6" t="n">
-        <v>506.6047800584543</v>
+        <v>503.9597395935223</v>
       </c>
       <c r="Q301" s="6" t="n">
-        <v>494.2130082270505</v>
+        <v>491.4770945834908</v>
       </c>
       <c r="R301" s="6" t="n">
-        <v>481.2967951729616</v>
+        <v>478.5042300823091</v>
       </c>
       <c r="S301" s="6" t="n">
-        <v>467.7443461066698</v>
+        <v>464.9271554519713</v>
       </c>
       <c r="T301" s="6" t="n">
-        <v>453.7925282911789</v>
+        <v>450.9803523296507</v>
       </c>
       <c r="U301" s="6" t="n">
-        <v>439.1989318557941</v>
+        <v>436.4217364127733</v>
       </c>
       <c r="V301" s="6" t="n">
-        <v>424.13991993927</v>
+        <v>421.4237557618857</v>
       </c>
       <c r="W301" s="6" t="n">
-        <v>408.0971134137725</v>
+        <v>405.4686313439784</v>
       </c>
       <c r="X301" s="6" t="n">
-        <v>391.5638881387553</v>
+        <v>389.0422073906283</v>
       </c>
       <c r="Y301" s="6" t="n">
-        <v>375.4895877220902</v>
+        <v>373.0965245445778</v>
       </c>
       <c r="Z301" s="6" t="n">
-        <v>359.4077235518013</v>
+        <v>357.1804959840188</v>
       </c>
       <c r="AA301" s="6" t="n">
-        <v>342.6596206375829</v>
+        <v>340.6275277253407</v>
       </c>
       <c r="AB301" s="6" t="n">
-        <v>325.4227660906203</v>
+        <v>323.6052651093041</v>
       </c>
       <c r="AC301" s="6" t="n">
-        <v>307.362433086384</v>
+        <v>305.7848448284669</v>
       </c>
       <c r="AD301" s="6" t="n">
-        <v>288.7037891303016</v>
+        <v>287.3807270505294</v>
       </c>
       <c r="AE301" s="6" t="n">
-        <v>268.3299115307742</v>
+        <v>267.2791093121773</v>
       </c>
       <c r="AF301" s="6" t="n">
-        <v>247.080353683255</v>
+        <v>246.3025522553589</v>
       </c>
       <c r="AG301" s="6" t="n">
-        <v>225.0853233737332</v>
+        <v>224.5856525862596</v>
       </c>
       <c r="AH301" s="6" t="n">
-        <v>202.6797950579354</v>
+        <v>202.4722302496085</v>
       </c>
       <c r="AI301" s="6" t="n">
-        <v>179.1494747074693</v>
+        <v>179.232461182222</v>
       </c>
       <c r="AJ301" s="6" t="n">
-        <v>154.9282448221257</v>
+        <v>155.2836495089831</v>
       </c>
       <c r="AK301" s="6" t="n">
-        <v>129.5376705544141</v>
+        <v>130.1512365715346</v>
       </c>
       <c r="AL301" s="6" t="n">
-        <v>103.3252483584307</v>
+        <v>104.1678182221423</v>
       </c>
       <c r="AM301" s="6" t="n">
-        <v>75.53120117391893</v>
+        <v>76.57207393723277</v>
       </c>
       <c r="AN301" s="6" t="n">
-        <v>47.15945564157511</v>
+        <v>48.10595692093149</v>
       </c>
       <c r="AO301" s="6" t="n">
-        <v>23.75310238699667</v>
+        <v>23.78452368804357</v>
       </c>
       <c r="AP301" s="6" t="n">
         <v>0</v>
@@ -7448,106 +7448,106 @@
         <v>0</v>
       </c>
       <c r="K309" s="6" t="n">
-        <v>72.03829474521896</v>
+        <v>71.66600088348895</v>
       </c>
       <c r="L309" s="6" t="n">
-        <v>73.51887276343012</v>
+        <v>73.13661140292268</v>
       </c>
       <c r="M309" s="6" t="n">
-        <v>75.40617553902828</v>
+        <v>75.01191436182141</v>
       </c>
       <c r="N309" s="6" t="n">
-        <v>78.07421473717562</v>
+        <v>77.66431772698481</v>
       </c>
       <c r="O309" s="6" t="n">
-        <v>81.91599308048065</v>
+        <v>81.48479486598529</v>
       </c>
       <c r="P309" s="6" t="n">
-        <v>87.21000268067854</v>
+        <v>86.75057095409854</v>
       </c>
       <c r="Q309" s="6" t="n">
-        <v>94.11618703202072</v>
+        <v>93.62109286393991</v>
       </c>
       <c r="R309" s="6" t="n">
-        <v>102.8823415907884</v>
+        <v>102.3424337527551</v>
       </c>
       <c r="S309" s="6" t="n">
-        <v>113.5022413334215</v>
+        <v>112.9087224737133</v>
       </c>
       <c r="T309" s="6" t="n">
-        <v>126.0097195597594</v>
+        <v>125.353413462763</v>
       </c>
       <c r="U309" s="6" t="n">
-        <v>140.2836182208805</v>
+        <v>139.5560811486539</v>
       </c>
       <c r="V309" s="6" t="n">
-        <v>156.2511438360465</v>
+        <v>155.4440229952658</v>
       </c>
       <c r="W309" s="6" t="n">
-        <v>173.7077024568702</v>
+        <v>172.8136949435213</v>
       </c>
       <c r="X309" s="6" t="n">
-        <v>192.4025609545302</v>
+        <v>191.4156366380475</v>
       </c>
       <c r="Y309" s="6" t="n">
-        <v>212.1224961922896</v>
+        <v>211.037368268875</v>
       </c>
       <c r="Z309" s="6" t="n">
-        <v>232.5249987992842</v>
+        <v>231.338225423894</v>
       </c>
       <c r="AA309" s="6" t="n">
-        <v>253.3550550829947</v>
+        <v>252.0641169680273</v>
       </c>
       <c r="AB309" s="6" t="n">
-        <v>274.9625112136583</v>
+        <v>273.5633491669572</v>
       </c>
       <c r="AC309" s="6" t="n">
-        <v>295.573347969675</v>
+        <v>294.0705657603964</v>
       </c>
       <c r="AD309" s="6" t="n">
-        <v>315.6942886417129</v>
+        <v>314.0894994948451</v>
       </c>
       <c r="AE309" s="6" t="n">
-        <v>334.9285707017309</v>
+        <v>333.2257427826887</v>
       </c>
       <c r="AF309" s="6" t="n">
-        <v>353.0762113009259</v>
+        <v>351.2799287307991</v>
       </c>
       <c r="AG309" s="6" t="n">
-        <v>369.8270855783692</v>
+        <v>367.9437632657763</v>
       </c>
       <c r="AH309" s="6" t="n">
-        <v>385.0658631524328</v>
+        <v>383.102103336144</v>
       </c>
       <c r="AI309" s="6" t="n">
-        <v>398.6100572520498</v>
+        <v>396.5735407491459</v>
       </c>
       <c r="AJ309" s="6" t="n">
-        <v>410.3341888433459</v>
+        <v>408.2334168264667</v>
       </c>
       <c r="AK309" s="6" t="n">
-        <v>420.3015849535684</v>
+        <v>418.1443894249751</v>
       </c>
       <c r="AL309" s="6" t="n">
-        <v>428.480478068478</v>
+        <v>426.2752805830067</v>
       </c>
       <c r="AM309" s="6" t="n">
-        <v>435.0832520222062</v>
+        <v>432.8370856977285</v>
       </c>
       <c r="AN309" s="6" t="n">
-        <v>440.2743361688925</v>
+        <v>437.9936851972857</v>
       </c>
       <c r="AO309" s="6" t="n">
-        <v>444.2027041636388</v>
+        <v>441.894042737951</v>
       </c>
       <c r="AP309" s="6" t="n">
-        <v>447.4816350572161</v>
+        <v>445.1472601202943</v>
       </c>
       <c r="AQ309" s="6" t="n">
-        <v>479.6249919693773</v>
+        <v>477.129138268712</v>
       </c>
       <c r="AR309" s="6" t="n">
-        <v>504.4002583438451</v>
+        <v>501.7767943702416</v>
       </c>
       <c r="AS309" s="6" t="n">
         <v>0</v>
@@ -25879,7 +25879,7 @@
     <row r="11">
       <c r="D11" t="inlineStr">
         <is>
-          <t>First installment share of remaining profile</t>
+          <t>First installment share of remaining profile (A, B, commercial, standby)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -25904,7 +25904,7 @@
         </is>
       </c>
       <c r="F12" s="11">
-        <f>$F$11+(INDEX(Operations!$J$9:$BN$9,1,Time!$F$13)+Inputs!$F$79)/100*INDEX(Time!$J$25:$BN$25,1,Time!$F$13)/Inputs!$F$247*1</f>
+        <f>INDEX(Debt!$J$147:$BN$147,1,Time!$F$13)+(INDEX(Operations!$J$9:$BN$9,1,Time!$F$13)+Inputs!$F$79)/100*INDEX(Time!$J$25:$BN$25,1,Time!$F$13)/Inputs!$F$247*1</f>
         <v/>
       </c>
     </row>
@@ -37648,7 +37648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN19"/>
+  <dimension ref="A1:BN147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -40708,6 +40708,733 @@
         <v/>
       </c>
     </row>
+    <row r="144">
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>ECA-covered tranche: contractual schedule (equal semiannual installments, first repayment period to final maturity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>ECA installment, share of the ECA amount</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="J145" s="11">
+        <f>IF(Time!J53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="K145" s="11">
+        <f>IF(Time!K53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="L145" s="11">
+        <f>IF(Time!L53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="M145" s="11">
+        <f>IF(Time!M53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="N145" s="11">
+        <f>IF(Time!N53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="O145" s="11">
+        <f>IF(Time!O53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="P145" s="11">
+        <f>IF(Time!P53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="Q145" s="11">
+        <f>IF(Time!Q53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="R145" s="11">
+        <f>IF(Time!R53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="S145" s="11">
+        <f>IF(Time!S53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="T145" s="11">
+        <f>IF(Time!T53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="U145" s="11">
+        <f>IF(Time!U53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="V145" s="11">
+        <f>IF(Time!V53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="W145" s="11">
+        <f>IF(Time!W53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="X145" s="11">
+        <f>IF(Time!X53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="Y145" s="11">
+        <f>IF(Time!Y53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="Z145" s="11">
+        <f>IF(Time!Z53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AA145" s="11">
+        <f>IF(Time!AA53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AB145" s="11">
+        <f>IF(Time!AB53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AC145" s="11">
+        <f>IF(Time!AC53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AD145" s="11">
+        <f>IF(Time!AD53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AE145" s="11">
+        <f>IF(Time!AE53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AF145" s="11">
+        <f>IF(Time!AF53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AG145" s="11">
+        <f>IF(Time!AG53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AH145" s="11">
+        <f>IF(Time!AH53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AI145" s="11">
+        <f>IF(Time!AI53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AJ145" s="11">
+        <f>IF(Time!AJ53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AK145" s="11">
+        <f>IF(Time!AK53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AL145" s="11">
+        <f>IF(Time!AL53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AM145" s="11">
+        <f>IF(Time!AM53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AN145" s="11">
+        <f>IF(Time!AN53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AO145" s="11">
+        <f>IF(Time!AO53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AP145" s="11">
+        <f>IF(Time!AP53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AQ145" s="11">
+        <f>IF(Time!AQ53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AR145" s="11">
+        <f>IF(Time!AR53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AS145" s="11">
+        <f>IF(Time!AS53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AT145" s="11">
+        <f>IF(Time!AT53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AU145" s="11">
+        <f>IF(Time!AU53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AV145" s="11">
+        <f>IF(Time!AV53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AW145" s="11">
+        <f>IF(Time!AW53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AX145" s="11">
+        <f>IF(Time!AX53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AY145" s="11">
+        <f>IF(Time!AY53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="AZ145" s="11">
+        <f>IF(Time!AZ53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BA145" s="11">
+        <f>IF(Time!BA53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BB145" s="11">
+        <f>IF(Time!BB53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BC145" s="11">
+        <f>IF(Time!BC53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BD145" s="11">
+        <f>IF(Time!BD53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BE145" s="11">
+        <f>IF(Time!BE53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BF145" s="11">
+        <f>IF(Time!BF53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BG145" s="11">
+        <f>IF(Time!BG53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BH145" s="11">
+        <f>IF(Time!BH53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BI145" s="11">
+        <f>IF(Time!BI53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BJ145" s="11">
+        <f>IF(Time!BJ53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BK145" s="11">
+        <f>IF(Time!BK53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BL145" s="11">
+        <f>IF(Time!BL53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BM145" s="11">
+        <f>IF(Time!BM53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+      <c r="BN145" s="11">
+        <f>IF(Time!BN53=1,1/SUM(Time!$J$53:$BN$53),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ECA remaining profile (this and later installments)</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="J146" s="11">
+        <f>SUM(J145:BN145)</f>
+        <v/>
+      </c>
+      <c r="K146" s="11">
+        <f>SUM(K145:BN145)</f>
+        <v/>
+      </c>
+      <c r="L146" s="11">
+        <f>SUM(L145:BN145)</f>
+        <v/>
+      </c>
+      <c r="M146" s="11">
+        <f>SUM(M145:BN145)</f>
+        <v/>
+      </c>
+      <c r="N146" s="11">
+        <f>SUM(N145:BN145)</f>
+        <v/>
+      </c>
+      <c r="O146" s="11">
+        <f>SUM(O145:BN145)</f>
+        <v/>
+      </c>
+      <c r="P146" s="11">
+        <f>SUM(P145:BN145)</f>
+        <v/>
+      </c>
+      <c r="Q146" s="11">
+        <f>SUM(Q145:BN145)</f>
+        <v/>
+      </c>
+      <c r="R146" s="11">
+        <f>SUM(R145:BN145)</f>
+        <v/>
+      </c>
+      <c r="S146" s="11">
+        <f>SUM(S145:BN145)</f>
+        <v/>
+      </c>
+      <c r="T146" s="11">
+        <f>SUM(T145:BN145)</f>
+        <v/>
+      </c>
+      <c r="U146" s="11">
+        <f>SUM(U145:BN145)</f>
+        <v/>
+      </c>
+      <c r="V146" s="11">
+        <f>SUM(V145:BN145)</f>
+        <v/>
+      </c>
+      <c r="W146" s="11">
+        <f>SUM(W145:BN145)</f>
+        <v/>
+      </c>
+      <c r="X146" s="11">
+        <f>SUM(X145:BN145)</f>
+        <v/>
+      </c>
+      <c r="Y146" s="11">
+        <f>SUM(Y145:BN145)</f>
+        <v/>
+      </c>
+      <c r="Z146" s="11">
+        <f>SUM(Z145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AA146" s="11">
+        <f>SUM(AA145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AB146" s="11">
+        <f>SUM(AB145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AC146" s="11">
+        <f>SUM(AC145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AD146" s="11">
+        <f>SUM(AD145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AE146" s="11">
+        <f>SUM(AE145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AF146" s="11">
+        <f>SUM(AF145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AG146" s="11">
+        <f>SUM(AG145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AH146" s="11">
+        <f>SUM(AH145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AI146" s="11">
+        <f>SUM(AI145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AJ146" s="11">
+        <f>SUM(AJ145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AK146" s="11">
+        <f>SUM(AK145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AL146" s="11">
+        <f>SUM(AL145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AM146" s="11">
+        <f>SUM(AM145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AN146" s="11">
+        <f>SUM(AN145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AO146" s="11">
+        <f>SUM(AO145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AP146" s="11">
+        <f>SUM(AP145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AQ146" s="11">
+        <f>SUM(AQ145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AR146" s="11">
+        <f>SUM(AR145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AS146" s="11">
+        <f>SUM(AS145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AT146" s="11">
+        <f>SUM(AT145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AU146" s="11">
+        <f>SUM(AU145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AV146" s="11">
+        <f>SUM(AV145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AW146" s="11">
+        <f>SUM(AW145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AX146" s="11">
+        <f>SUM(AX145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AY146" s="11">
+        <f>SUM(AY145:BN145)</f>
+        <v/>
+      </c>
+      <c r="AZ146" s="11">
+        <f>SUM(AZ145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BA146" s="11">
+        <f>SUM(BA145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BB146" s="11">
+        <f>SUM(BB145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BC146" s="11">
+        <f>SUM(BC145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BD146" s="11">
+        <f>SUM(BD145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BE146" s="11">
+        <f>SUM(BE145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BF146" s="11">
+        <f>SUM(BF145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BG146" s="11">
+        <f>SUM(BG145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BH146" s="11">
+        <f>SUM(BH145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BI146" s="11">
+        <f>SUM(BI145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BJ146" s="11">
+        <f>SUM(BJ145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BK146" s="11">
+        <f>SUM(BK145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BL146" s="11">
+        <f>SUM(BL145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BM146" s="11">
+        <f>SUM(BM145:BN145)</f>
+        <v/>
+      </c>
+      <c r="BN146" s="11">
+        <f>SUM(BN145:BN145)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>ECA installment share of remaining balance</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="J147" s="11">
+        <f>IF(J146&gt;Inputs!$F$253,J145/J146,0)</f>
+        <v/>
+      </c>
+      <c r="K147" s="11">
+        <f>IF(K146&gt;Inputs!$F$253,K145/K146,0)</f>
+        <v/>
+      </c>
+      <c r="L147" s="11">
+        <f>IF(L146&gt;Inputs!$F$253,L145/L146,0)</f>
+        <v/>
+      </c>
+      <c r="M147" s="11">
+        <f>IF(M146&gt;Inputs!$F$253,M145/M146,0)</f>
+        <v/>
+      </c>
+      <c r="N147" s="11">
+        <f>IF(N146&gt;Inputs!$F$253,N145/N146,0)</f>
+        <v/>
+      </c>
+      <c r="O147" s="11">
+        <f>IF(O146&gt;Inputs!$F$253,O145/O146,0)</f>
+        <v/>
+      </c>
+      <c r="P147" s="11">
+        <f>IF(P146&gt;Inputs!$F$253,P145/P146,0)</f>
+        <v/>
+      </c>
+      <c r="Q147" s="11">
+        <f>IF(Q146&gt;Inputs!$F$253,Q145/Q146,0)</f>
+        <v/>
+      </c>
+      <c r="R147" s="11">
+        <f>IF(R146&gt;Inputs!$F$253,R145/R146,0)</f>
+        <v/>
+      </c>
+      <c r="S147" s="11">
+        <f>IF(S146&gt;Inputs!$F$253,S145/S146,0)</f>
+        <v/>
+      </c>
+      <c r="T147" s="11">
+        <f>IF(T146&gt;Inputs!$F$253,T145/T146,0)</f>
+        <v/>
+      </c>
+      <c r="U147" s="11">
+        <f>IF(U146&gt;Inputs!$F$253,U145/U146,0)</f>
+        <v/>
+      </c>
+      <c r="V147" s="11">
+        <f>IF(V146&gt;Inputs!$F$253,V145/V146,0)</f>
+        <v/>
+      </c>
+      <c r="W147" s="11">
+        <f>IF(W146&gt;Inputs!$F$253,W145/W146,0)</f>
+        <v/>
+      </c>
+      <c r="X147" s="11">
+        <f>IF(X146&gt;Inputs!$F$253,X145/X146,0)</f>
+        <v/>
+      </c>
+      <c r="Y147" s="11">
+        <f>IF(Y146&gt;Inputs!$F$253,Y145/Y146,0)</f>
+        <v/>
+      </c>
+      <c r="Z147" s="11">
+        <f>IF(Z146&gt;Inputs!$F$253,Z145/Z146,0)</f>
+        <v/>
+      </c>
+      <c r="AA147" s="11">
+        <f>IF(AA146&gt;Inputs!$F$253,AA145/AA146,0)</f>
+        <v/>
+      </c>
+      <c r="AB147" s="11">
+        <f>IF(AB146&gt;Inputs!$F$253,AB145/AB146,0)</f>
+        <v/>
+      </c>
+      <c r="AC147" s="11">
+        <f>IF(AC146&gt;Inputs!$F$253,AC145/AC146,0)</f>
+        <v/>
+      </c>
+      <c r="AD147" s="11">
+        <f>IF(AD146&gt;Inputs!$F$253,AD145/AD146,0)</f>
+        <v/>
+      </c>
+      <c r="AE147" s="11">
+        <f>IF(AE146&gt;Inputs!$F$253,AE145/AE146,0)</f>
+        <v/>
+      </c>
+      <c r="AF147" s="11">
+        <f>IF(AF146&gt;Inputs!$F$253,AF145/AF146,0)</f>
+        <v/>
+      </c>
+      <c r="AG147" s="11">
+        <f>IF(AG146&gt;Inputs!$F$253,AG145/AG146,0)</f>
+        <v/>
+      </c>
+      <c r="AH147" s="11">
+        <f>IF(AH146&gt;Inputs!$F$253,AH145/AH146,0)</f>
+        <v/>
+      </c>
+      <c r="AI147" s="11">
+        <f>IF(AI146&gt;Inputs!$F$253,AI145/AI146,0)</f>
+        <v/>
+      </c>
+      <c r="AJ147" s="11">
+        <f>IF(AJ146&gt;Inputs!$F$253,AJ145/AJ146,0)</f>
+        <v/>
+      </c>
+      <c r="AK147" s="11">
+        <f>IF(AK146&gt;Inputs!$F$253,AK145/AK146,0)</f>
+        <v/>
+      </c>
+      <c r="AL147" s="11">
+        <f>IF(AL146&gt;Inputs!$F$253,AL145/AL146,0)</f>
+        <v/>
+      </c>
+      <c r="AM147" s="11">
+        <f>IF(AM146&gt;Inputs!$F$253,AM145/AM146,0)</f>
+        <v/>
+      </c>
+      <c r="AN147" s="11">
+        <f>IF(AN146&gt;Inputs!$F$253,AN145/AN146,0)</f>
+        <v/>
+      </c>
+      <c r="AO147" s="11">
+        <f>IF(AO146&gt;Inputs!$F$253,AO145/AO146,0)</f>
+        <v/>
+      </c>
+      <c r="AP147" s="11">
+        <f>IF(AP146&gt;Inputs!$F$253,AP145/AP146,0)</f>
+        <v/>
+      </c>
+      <c r="AQ147" s="11">
+        <f>IF(AQ146&gt;Inputs!$F$253,AQ145/AQ146,0)</f>
+        <v/>
+      </c>
+      <c r="AR147" s="11">
+        <f>IF(AR146&gt;Inputs!$F$253,AR145/AR146,0)</f>
+        <v/>
+      </c>
+      <c r="AS147" s="11">
+        <f>IF(AS146&gt;Inputs!$F$253,AS145/AS146,0)</f>
+        <v/>
+      </c>
+      <c r="AT147" s="11">
+        <f>IF(AT146&gt;Inputs!$F$253,AT145/AT146,0)</f>
+        <v/>
+      </c>
+      <c r="AU147" s="11">
+        <f>IF(AU146&gt;Inputs!$F$253,AU145/AU146,0)</f>
+        <v/>
+      </c>
+      <c r="AV147" s="11">
+        <f>IF(AV146&gt;Inputs!$F$253,AV145/AV146,0)</f>
+        <v/>
+      </c>
+      <c r="AW147" s="11">
+        <f>IF(AW146&gt;Inputs!$F$253,AW145/AW146,0)</f>
+        <v/>
+      </c>
+      <c r="AX147" s="11">
+        <f>IF(AX146&gt;Inputs!$F$253,AX145/AX146,0)</f>
+        <v/>
+      </c>
+      <c r="AY147" s="11">
+        <f>IF(AY146&gt;Inputs!$F$253,AY145/AY146,0)</f>
+        <v/>
+      </c>
+      <c r="AZ147" s="11">
+        <f>IF(AZ146&gt;Inputs!$F$253,AZ145/AZ146,0)</f>
+        <v/>
+      </c>
+      <c r="BA147" s="11">
+        <f>IF(BA146&gt;Inputs!$F$253,BA145/BA146,0)</f>
+        <v/>
+      </c>
+      <c r="BB147" s="11">
+        <f>IF(BB146&gt;Inputs!$F$253,BB145/BB146,0)</f>
+        <v/>
+      </c>
+      <c r="BC147" s="11">
+        <f>IF(BC146&gt;Inputs!$F$253,BC145/BC146,0)</f>
+        <v/>
+      </c>
+      <c r="BD147" s="11">
+        <f>IF(BD146&gt;Inputs!$F$253,BD145/BD146,0)</f>
+        <v/>
+      </c>
+      <c r="BE147" s="11">
+        <f>IF(BE146&gt;Inputs!$F$253,BE145/BE146,0)</f>
+        <v/>
+      </c>
+      <c r="BF147" s="11">
+        <f>IF(BF146&gt;Inputs!$F$253,BF145/BF146,0)</f>
+        <v/>
+      </c>
+      <c r="BG147" s="11">
+        <f>IF(BG146&gt;Inputs!$F$253,BG145/BG146,0)</f>
+        <v/>
+      </c>
+      <c r="BH147" s="11">
+        <f>IF(BH146&gt;Inputs!$F$253,BH145/BH146,0)</f>
+        <v/>
+      </c>
+      <c r="BI147" s="11">
+        <f>IF(BI146&gt;Inputs!$F$253,BI145/BI146,0)</f>
+        <v/>
+      </c>
+      <c r="BJ147" s="11">
+        <f>IF(BJ146&gt;Inputs!$F$253,BJ145/BJ146,0)</f>
+        <v/>
+      </c>
+      <c r="BK147" s="11">
+        <f>IF(BK146&gt;Inputs!$F$253,BK145/BK146,0)</f>
+        <v/>
+      </c>
+      <c r="BL147" s="11">
+        <f>IF(BL146&gt;Inputs!$F$253,BL145/BL146,0)</f>
+        <v/>
+      </c>
+      <c r="BM147" s="11">
+        <f>IF(BM146&gt;Inputs!$F$253,BM145/BM146,0)</f>
+        <v/>
+      </c>
+      <c r="BN147" s="11">
+        <f>IF(BN146&gt;Inputs!$F$253,BN145/BN146,0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>